<commit_message>
Make escape puzzles clear and reusable across subjects
Allow subject devices in all P1–P8 slots, add science and Korean examples, and show how each clue maps to its input. Replace arbitrary flips with candidate matching, provide a numeric keypad, and update the teacher workbook and authoring prompt.

Validated 43 first-love tests, XLSX image import, custom lessons through the service, and desktop/mobile UI flows.
</commit_message>
<xml_diff>
--- a/public/labs/first-love/first-love-template-v3.xlsx
+++ b/public/labs/first-love/first-love-template-v3.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="Rc95d7197a9984d06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R573a8aeb66b5475a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="R839663107c934953"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="Rac252a050f06464a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R57d89cca232f49d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="Rb493126ca429463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R6f2f83a8282748a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R50ca6286049b4d2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="R0d93641f74b5403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="R857002d605b9494a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R973903099b484dfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R12c379eec1e442eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -107,6 +107,173 @@
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1524000" cy="1066800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="aa4cdcc4-fb32-4522-8b02-7c690cc36b60"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcad604df1482440d"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1524000" cy="1066800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="9c91fa75-fb00-401c-9d84-64ff1d9a6916"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R08900cffe60a4687"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1524000" cy="1066800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="b6d4010a-eba3-4784-af86-2b9cb0f5168b"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd7416cbf4aae4029"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1524000" cy="1066800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="f16327c3-8d19-4e7b-b9e8-3669dda30981"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc8bc48c058384cbb"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1524000" cy="1066800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="50de4ea1-f5f8-4ac6-8d85-068c4656f180"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R62beb618026d400a"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1524000" cy="1066800"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="3cf85678-147a-4664-a939-7abc8f4c0f97"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2cb68e4d3fa14dd7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -352,7 +519,7 @@
         <x:v>과목</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>협동 시연</x:v>
+        <x:v>과학 예시</x:v>
       </x:c>
       <x:c r="C7" s="4" t="str">
         <x:v>교사 입력</x:v>
@@ -363,7 +530,7 @@
         <x:v>단원</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>축제 방탈출 부스 · 교과 자료 교체 가능</x:v>
+        <x:v>물질의 구성 · 소화계</x:v>
       </x:c>
       <x:c r="C8" s="4" t="str">
         <x:v>교사 입력</x:v>
@@ -374,7 +541,7 @@
         <x:v>대상</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>공통</x:v>
+        <x:v>중학교 예시</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
         <x:v>교사 입력</x:v>
@@ -427,6 +594,12 @@
       <x:c r="A2" s="5" t="str">
         <x:v>퍼즐 · 오늘, 너에게 v3</x:v>
       </x:c>
+      <x:c r="D2" t="str">
+        <x:v>P1~P8 교과 교체 가능</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>형식을 바꾸고 자료·대상·단서를 작성하세요.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="8" t="str">
@@ -467,7 +640,7 @@
       <x:c r="B5" s="4" t="str">
         <x:v>classroom</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="str">
+      <x:c r="C5" s="9" t="str">
         <x:v>riddle</x:v>
       </x:c>
       <x:c r="D5" s="4" t="str">
@@ -499,7 +672,7 @@
       <x:c r="B6" s="4" t="str">
         <x:v>classroom</x:v>
       </x:c>
-      <x:c r="C6" s="4" t="str">
+      <x:c r="C6" s="9" t="str">
         <x:v>jigsaw</x:v>
       </x:c>
       <x:c r="D6" s="4" t="str">
@@ -531,29 +704,29 @@
       <x:c r="B7" s="4" t="str">
         <x:v>library</x:v>
       </x:c>
-      <x:c r="C7" s="4" t="str">
+      <x:c r="C7" s="9" t="str">
         <x:v>dials</x:v>
       </x:c>
-      <x:c r="D7" s="4" t="str">
-        <x:v>도서관의 작은 도구함</x:v>
+      <x:c r="D7" s="9" t="str">
+        <x:v>분자식이 남긴 네 자리 암호</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>네 다이얼을 맞춘 뒤 손잡이를 당기세요.</x:v>
+        <x:v>각 기록의 원소를 찾고, 번호표의 숫자 네 개로 도구함을 여세요.</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
-        <x:v>축제 부스의 시연 자료 · 친구가 찾은 기록을 서로 알려 주세요.</x:v>
+        <x:v>기록 1~4는 암호 1~4에 대응합니다. 번호표의 숫자를 입력하세요.</x:v>
       </x:c>
       <x:c r="G7" s="9" t="str">
-        <x:v>각 역할이 찾은 자료를 해당 번호의 장치에 적용합니다. 다른 역할의 기록만으로는 그 번호의 답을 알 수 없습니다.</x:v>
+        <x:v>H₂O에서 H 원자 2개, CO₂에서 C 원자 1개, O₂는 산소, N₂는 질소. 번호표에서 H=3, C=5, O=2, N=6이므로 암호는 3526이다. 각 기록은 독립된 한 자리의 원소를 지정하므로 한 기록이 없으면 그 자리는 여러 숫자가 가능하다.</x:v>
       </x:c>
       <x:c r="H7" s="9" t="str">
-        <x:v>각자 주변에서 기록을 찾아 단서함을 펼쳐 보세요.</x:v>
+        <x:v>내 역할이 표시된 주변 사물에서 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I7" s="9" t="str">
-        <x:v>단서의 번호와 장치의 번호를 맞춰 비교하세요.</x:v>
+        <x:v>기록이 가리키는 대상을 자료와 비교하세요. 같은 번호의 입력칸에 사용합니다.</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
-        <x:v>전부 맞춘 뒤 아래 버튼으로 한 번에 확인하세요.</x:v>
+        <x:v>네 칸을 모두 채운 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="90" customHeight="1">
@@ -563,29 +736,29 @@
       <x:c r="B8" s="4" t="str">
         <x:v>library</x:v>
       </x:c>
-      <x:c r="C8" s="4" t="str">
+      <x:c r="C8" s="9" t="str">
         <x:v>circuit</x:v>
       </x:c>
-      <x:c r="D8" s="4" t="str">
-        <x:v>전원이 닿는 곳</x:v>
+      <x:c r="D8" s="9" t="str">
+        <x:v>소화 기록과 효소 연결하기</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>커넥터를 꽂고 네 선을 연결한 뒤 전원을 넣으세요.</x:v>
+        <x:v>각 기록에서 작용한 효소를 찾아 네 연결선을 이으세요.</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
-        <x:v>축제 부스의 시연 자료 · 친구가 찾은 기록을 서로 알려 주세요.</x:v>
+        <x:v>왼쪽 연결선과 같은 번호의 단서를 읽고, 오른쪽 효소에 연결하세요.</x:v>
       </x:c>
       <x:c r="G8" s="9" t="str">
-        <x:v>각 역할이 찾은 자료를 해당 번호의 장치에 적용합니다. 다른 역할의 기록만으로는 그 번호의 답을 알 수 없습니다.</x:v>
+        <x:v>침의 아밀레이스는 녹말, 위액의 펩신은 단백질, 이자액의 리파아제는 지방, 트립신은 단백질을 분해한다. 쓸개즙은 소화 효소가 아니다. 각 단서를 빼면 해당 선의 대상이 정해지지 않는다. 같은 대상에 여러 선을 연결할 수 있으므로 남은 단자만으로 추론할 수 없다.</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
-        <x:v>각자 주변에서 기록을 찾아 단서함을 펼쳐 보세요.</x:v>
+        <x:v>내 역할이 표시된 주변 사물에서 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I8" s="9" t="str">
-        <x:v>단서의 번호와 장치의 번호를 맞춰 비교하세요.</x:v>
+        <x:v>기록이 가리키는 대상을 자료와 비교하세요. 같은 번호의 입력칸에 사용합니다.</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>전부 맞춘 뒤 아래 버튼으로 한 번에 확인하세요.</x:v>
+        <x:v>네 칸을 모두 채운 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="90" customHeight="1">
@@ -595,7 +768,7 @@
       <x:c r="B9" s="4" t="str">
         <x:v>club</x:v>
       </x:c>
-      <x:c r="C9" s="4" t="str">
+      <x:c r="C9" s="9" t="str">
         <x:v>tools</x:v>
       </x:c>
       <x:c r="D9" s="4" t="str">
@@ -627,7 +800,7 @@
       <x:c r="B10" s="4" t="str">
         <x:v>club</x:v>
       </x:c>
-      <x:c r="C10" s="4" t="str">
+      <x:c r="C10" s="9" t="str">
         <x:v>film</x:v>
       </x:c>
       <x:c r="D10" s="4" t="str">
@@ -659,29 +832,29 @@
       <x:c r="B11" s="4" t="str">
         <x:v>corridor</x:v>
       </x:c>
-      <x:c r="C11" s="4" t="str">
+      <x:c r="C11" s="9" t="str">
         <x:v>frames</x:v>
       </x:c>
-      <x:c r="D11" s="4" t="str">
-        <x:v>뒤섞인 전시판</x:v>
+      <x:c r="D11" s="9" t="str">
+        <x:v>입자 모형 전시판 복원하기</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>슬라이드를 액자에 끼우고 뒤집어 그림판을 닫으세요.</x:v>
+        <x:v>기록과 맞는 모형 네 장을 골라 같은 번호의 칸에 놓으세요.</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
-        <x:v>축제 부스의 시연 자료 · 친구가 찾은 기록을 서로 알려 주세요.</x:v>
+        <x:v>모형 안의 글자는 원소 기호입니다. 쓰지 않는 그림 두 장이 있습니다.</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
-        <x:v>각 역할이 찾은 자료를 해당 번호의 장치에 적용합니다. 다른 역할의 기록만으로는 그 번호의 답을 알 수 없습니다.</x:v>
+        <x:v>1=가(H₂), 2=다(H₂O), 3=라(CO₂), 4=마(He). 나(O₂), 바(O₃)는 사용하지 않는다. 원소의 종류와 원자 수를 함께 비교한다. 어느 단서를 빼도 미사용 그림과 그 칸의 그림을 바꾼 답이 추가로 가능하다.</x:v>
       </x:c>
       <x:c r="H11" s="9" t="str">
-        <x:v>각자 주변에서 기록을 찾아 단서함을 펼쳐 보세요.</x:v>
+        <x:v>내 역할이 표시된 주변 사물에서 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:v>단서의 번호와 장치의 번호를 맞춰 비교하세요.</x:v>
+        <x:v>기록이 가리키는 대상을 자료와 비교하세요. 같은 번호의 입력칸에 사용합니다.</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
-        <x:v>전부 맞춘 뒤 아래 버튼으로 한 번에 확인하세요.</x:v>
+        <x:v>네 칸을 모두 채운 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="90" customHeight="1">
@@ -691,32 +864,58 @@
       <x:c r="B12" s="4" t="str">
         <x:v>corridor</x:v>
       </x:c>
-      <x:c r="C12" s="4" t="str">
+      <x:c r="C12" s="9" t="str">
         <x:v>key</x:v>
       </x:c>
-      <x:c r="D12" s="4" t="str">
-        <x:v>네가 하려던 말</x:v>
+      <x:c r="D12" s="9" t="str">
+        <x:v>소화 기관 열쇠 맞추기</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>열쇠 조각의 자리와 앞뒤를 맞춘 뒤 합치세요.</x:v>
+        <x:v>네 기록이 가리키는 기관 조각을 찾아 열쇠홈에 끼우세요.</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str">
-        <x:v>축제 부스의 시연 자료 · 친구가 찾은 기록을 서로 알려 주세요.</x:v>
+        <x:v>홈 번호는 기록 번호입니다. 음식이 지나가는 순서를 묻는 문제가 아닙니다.</x:v>
       </x:c>
       <x:c r="G12" s="9" t="str">
-        <x:v>각 역할이 찾은 자료를 해당 번호의 장치에 적용합니다. 다른 역할의 기록만으로는 그 번호의 답을 알 수 없습니다.</x:v>
+        <x:v>1=위, 2=입, 3=작은창자, 4=큰창자. 식도와 간 조각은 사용하지 않는다. 기능과 기관을 대응하며 임의의 회전·앞뒤 조건은 없다. 단서 하나가 빠지면 그 칸과 두 미사용 조각 중 무엇을 선택할지 정할 수 없다.</x:v>
       </x:c>
       <x:c r="H12" s="9" t="str">
-        <x:v>각자 주변에서 기록을 찾아 단서함을 펼쳐 보세요.</x:v>
+        <x:v>내 역할이 표시된 주변 사물에서 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I12" s="9" t="str">
-        <x:v>단서의 번호와 장치의 번호를 맞춰 비교하세요.</x:v>
+        <x:v>기록이 가리키는 대상을 자료와 비교하세요. 같은 번호의 입력칸에 사용합니다.</x:v>
       </x:c>
       <x:c r="J12" s="9" t="str">
-        <x:v>전부 맞춘 뒤 아래 버튼으로 한 번에 확인하세요.</x:v>
+        <x:v>네 칸을 모두 채운 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="8">
+    <x:dataValidation type="list" sqref="C5">
+      <x:formula1>"dials,circuit,frames,key,riddle"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C6">
+      <x:formula1>"dials,circuit,frames,key,jigsaw"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C7">
+      <x:formula1>"dials,circuit,frames,key"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C8">
+      <x:formula1>"dials,circuit,frames,key"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C9">
+      <x:formula1>"dials,circuit,frames,key,tools"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C10">
+      <x:formula1>"dials,circuit,frames,key,film"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C11">
+      <x:formula1>"dials,circuit,frames,key"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C12">
+      <x:formula1>"dials,circuit,frames,key"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -734,7 +933,7 @@
     <x:col min="7" max="7" width="11.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="11.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="14.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="25.559999465942383" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -886,7 +1085,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>□</x:v>
+        <x:v>철 Fe</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str"/>
       <x:c r="E9" s="4" t="n">
@@ -907,14 +1106,14 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>○</x:v>
+        <x:v>산소 O</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str"/>
       <x:c r="E10" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G10" s="4" t="str"/>
       <x:c r="H10" s="4" t="str"/>
@@ -930,14 +1129,14 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>△</x:v>
+        <x:v>수소 H</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str"/>
       <x:c r="E11" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G11" s="4" t="str"/>
       <x:c r="H11" s="4" t="str"/>
@@ -953,15 +1152,13 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>★</x:v>
+        <x:v>구리 Cu</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str"/>
       <x:c r="E12" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F12" s="9" t="str">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="F12" s="9" t="str"/>
       <x:c r="G12" s="4" t="str"/>
       <x:c r="H12" s="4" t="str"/>
       <x:c r="I12" s="4" t="str"/>
@@ -976,14 +1173,14 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>☾</x:v>
+        <x:v>탄소 C</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str"/>
       <x:c r="E13" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="9" t="str">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G13" s="4" t="str"/>
       <x:c r="H13" s="4" t="str"/>
@@ -999,13 +1196,15 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>♡</x:v>
+        <x:v>질소 N</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str"/>
       <x:c r="E14" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F14" s="9" t="str"/>
+      <x:c r="F14" s="9" t="str">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="G14" s="4" t="str"/>
       <x:c r="H14" s="4" t="str"/>
       <x:c r="I14" s="4" t="str"/>
@@ -1020,7 +1219,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>독서등</x:v>
+        <x:v>아밀레이스</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str"/>
       <x:c r="E15" s="4" t="n">
@@ -1043,7 +1242,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>환풍기</x:v>
+        <x:v>펩신</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str"/>
       <x:c r="E16" s="4" t="n">
@@ -1066,7 +1265,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>방송 스피커</x:v>
+        <x:v>리파아제</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str"/>
       <x:c r="E17" s="4" t="n">
@@ -1089,13 +1288,15 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>전시 조명</x:v>
+        <x:v>트립신</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str"/>
       <x:c r="E18" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F18" s="9" t="str"/>
+      <x:c r="F18" s="9" t="str">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="G18" s="4" t="str"/>
       <x:c r="H18" s="4" t="str"/>
       <x:c r="I18" s="4" t="str"/>
@@ -1110,7 +1311,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>분수 모터</x:v>
+        <x:v>쓸개즙</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str"/>
       <x:c r="E19" s="4" t="n">
@@ -1123,63 +1324,65 @@
       <x:c r="J19" s="9" t="str"/>
       <x:c r="K19" s="9" t="str"/>
     </x:row>
-    <x:row r="20" ht="45" customHeight="1">
+    <x:row r="20" ht="90" customHeight="1">
       <x:c r="A20" s="4" t="str">
-        <x:v>P4</x:v>
+        <x:v>P7</x:v>
       </x:c>
       <x:c r="B20" s="4" t="str">
-        <x:v>F</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>전광판</x:v>
+        <x:v>모형 가</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str"/>
       <x:c r="E20" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G20" s="4" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="str"/>
       <x:c r="H20" s="4" t="str"/>
       <x:c r="I20" s="4" t="str"/>
       <x:c r="J20" s="9" t="str"/>
-      <x:c r="K20" s="9" t="str"/>
-    </x:row>
-    <x:row r="21" ht="45" customHeight="1">
+      <x:c r="K20" s="9" t="str">
+        <x:v>원소 기호가 표시된 입자 모형 A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="90" customHeight="1">
       <x:c r="A21" s="4" t="str">
         <x:v>P7</x:v>
       </x:c>
       <x:c r="B21" s="4" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>새싹</x:v>
+        <x:v>모형 나</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str"/>
       <x:c r="E21" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="9" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G21" s="9" t="str">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>제외</x:v>
+      </x:c>
+      <x:c r="G21" s="9" t="str"/>
       <x:c r="H21" s="4" t="str"/>
       <x:c r="I21" s="4" t="str"/>
       <x:c r="J21" s="9" t="str"/>
-      <x:c r="K21" s="9" t="str"/>
-    </x:row>
-    <x:row r="22" ht="45" customHeight="1">
+      <x:c r="K21" s="9" t="str">
+        <x:v>원소 기호가 표시된 입자 모형 B</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="90" customHeight="1">
       <x:c r="A22" s="4" t="str">
         <x:v>P7</x:v>
       </x:c>
       <x:c r="B22" s="4" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>우산</x:v>
+        <x:v>모형 다</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str"/>
       <x:c r="E22" s="4" t="n">
@@ -1188,23 +1391,23 @@
       <x:c r="F22" s="9" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G22" s="9" t="str">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="G22" s="9" t="str"/>
       <x:c r="H22" s="4" t="str"/>
       <x:c r="I22" s="4" t="str"/>
       <x:c r="J22" s="9" t="str"/>
-      <x:c r="K22" s="9" t="str"/>
-    </x:row>
-    <x:row r="23" ht="45" customHeight="1">
+      <x:c r="K22" s="9" t="str">
+        <x:v>원소 기호가 표시된 입자 모형 C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="90" customHeight="1">
       <x:c r="A23" s="4" t="str">
         <x:v>P7</x:v>
       </x:c>
       <x:c r="B23" s="4" t="str">
-        <x:v>C</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
-        <x:v>눈사람</x:v>
+        <x:v>모형 라</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str"/>
       <x:c r="E23" s="4" t="n">
@@ -1213,23 +1416,23 @@
       <x:c r="F23" s="9" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="G23" s="9" t="str">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="G23" s="9" t="str"/>
       <x:c r="H23" s="4" t="str"/>
       <x:c r="I23" s="4" t="str"/>
       <x:c r="J23" s="9" t="str"/>
-      <x:c r="K23" s="9" t="str"/>
-    </x:row>
-    <x:row r="24" ht="45" customHeight="1">
+      <x:c r="K23" s="9" t="str">
+        <x:v>원소 기호가 표시된 입자 모형 D</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="90" customHeight="1">
       <x:c r="A24" s="4" t="str">
         <x:v>P7</x:v>
       </x:c>
       <x:c r="B24" s="4" t="str">
-        <x:v>D</x:v>
+        <x:v>E</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>나뭇잎</x:v>
+        <x:v>모형 마</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str"/>
       <x:c r="E24" s="4" t="n">
@@ -1238,23 +1441,23 @@
       <x:c r="F24" s="9" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G24" s="9" t="str">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="G24" s="9" t="str"/>
       <x:c r="H24" s="4" t="str"/>
       <x:c r="I24" s="4" t="str"/>
       <x:c r="J24" s="9" t="str"/>
-      <x:c r="K24" s="9" t="str"/>
-    </x:row>
-    <x:row r="25" ht="45" customHeight="1">
+      <x:c r="K24" s="9" t="str">
+        <x:v>원소 기호가 표시된 입자 모형 E</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="90" customHeight="1">
       <x:c r="A25" s="4" t="str">
         <x:v>P7</x:v>
       </x:c>
       <x:c r="B25" s="4" t="str">
-        <x:v>E</x:v>
+        <x:v>F</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>모래성</x:v>
+        <x:v>모형 바</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str"/>
       <x:c r="E25" s="4" t="n">
@@ -1263,34 +1466,32 @@
       <x:c r="F25" s="9" t="str">
         <x:v>제외</x:v>
       </x:c>
-      <x:c r="G25" s="9" t="str">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="G25" s="9" t="str"/>
       <x:c r="H25" s="4" t="str"/>
       <x:c r="I25" s="4" t="str"/>
       <x:c r="J25" s="9" t="str"/>
-      <x:c r="K25" s="9" t="str"/>
+      <x:c r="K25" s="9" t="str">
+        <x:v>원소 기호가 표시된 입자 모형 F</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="45" customHeight="1">
       <x:c r="A26" s="4" t="str">
-        <x:v>P7</x:v>
+        <x:v>P8</x:v>
       </x:c>
       <x:c r="B26" s="4" t="str">
-        <x:v>F</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>연</x:v>
+        <x:v>입</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str"/>
       <x:c r="E26" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F26" s="9" t="str">
-        <x:v>제외</x:v>
-      </x:c>
-      <x:c r="G26" s="9" t="str">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="str"/>
       <x:c r="H26" s="4" t="str"/>
       <x:c r="I26" s="4" t="str"/>
       <x:c r="J26" s="9" t="str"/>
@@ -1301,21 +1502,19 @@
         <x:v>P8</x:v>
       </x:c>
       <x:c r="B27" s="4" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
-        <x:v>○ 조각</x:v>
+        <x:v>위</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str"/>
       <x:c r="E27" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F27" s="9" t="str">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G27" s="9" t="str">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="G27" s="9" t="str"/>
       <x:c r="H27" s="4" t="str"/>
       <x:c r="I27" s="4" t="str"/>
       <x:c r="J27" s="9" t="str"/>
@@ -1326,21 +1525,19 @@
         <x:v>P8</x:v>
       </x:c>
       <x:c r="B28" s="4" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>△ 조각</x:v>
+        <x:v>작은창자</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str"/>
       <x:c r="E28" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F28" s="9" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G28" s="9" t="str">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G28" s="9" t="str"/>
       <x:c r="H28" s="4" t="str"/>
       <x:c r="I28" s="4" t="str"/>
       <x:c r="J28" s="9" t="str"/>
@@ -1351,21 +1548,19 @@
         <x:v>P8</x:v>
       </x:c>
       <x:c r="B29" s="4" t="str">
-        <x:v>C</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>□ 조각</x:v>
+        <x:v>큰창자</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str"/>
       <x:c r="E29" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F29" s="9" t="str">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G29" s="9" t="str">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G29" s="9" t="str"/>
       <x:c r="H29" s="4" t="str"/>
       <x:c r="I29" s="4" t="str"/>
       <x:c r="J29" s="9" t="str"/>
@@ -1376,28 +1571,50 @@
         <x:v>P8</x:v>
       </x:c>
       <x:c r="B30" s="4" t="str">
-        <x:v>D</x:v>
+        <x:v>E</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>★ 조각</x:v>
+        <x:v>식도</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str"/>
       <x:c r="E30" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F30" s="9" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G30" s="9" t="str">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>제외</x:v>
+      </x:c>
+      <x:c r="G30" s="9" t="str"/>
       <x:c r="H30" s="4" t="str"/>
       <x:c r="I30" s="4" t="str"/>
       <x:c r="J30" s="9" t="str"/>
       <x:c r="K30" s="9" t="str"/>
     </x:row>
+    <x:row r="31" ht="45" customHeight="1">
+      <x:c r="A31" s="4" t="str">
+        <x:v>P8</x:v>
+      </x:c>
+      <x:c r="B31" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C31" s="9" t="str">
+        <x:v>간</x:v>
+      </x:c>
+      <x:c r="D31" s="9" t="str"/>
+      <x:c r="E31" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F31" s="9" t="str">
+        <x:v>제외</x:v>
+      </x:c>
+      <x:c r="G31" s="9" t="str"/>
+      <x:c r="H31" s="4" t="str"/>
+      <x:c r="I31" s="4" t="str"/>
+      <x:c r="J31" s="9" t="str"/>
+      <x:c r="K31" s="9" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re067af41d8cc41c0"/>
 </x:worksheet>
 </file>
 
@@ -1416,6 +1633,14 @@
         <x:v>대상 · 오늘, 너에게 v3</x:v>
       </x:c>
     </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>역할 번호 = T1~T4</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>화면의 입력칸 이름</x:v>
+      </x:c>
+    </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="8" t="str">
         <x:v>퍼즐ID</x:v>
@@ -1428,6 +1653,230 @@
       </x:c>
       <x:c r="D4" s="8" t="str">
         <x:v>표시이름</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="45" customHeight="1">
+      <x:c r="A5" s="4" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>T1</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="str">
+        <x:v>암호 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="45" customHeight="1">
+      <x:c r="A6" s="4" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>T2</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
+        <x:v>암호 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="45" customHeight="1">
+      <x:c r="A7" s="4" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>T3</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="str">
+        <x:v>암호 3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="45" customHeight="1">
+      <x:c r="A8" s="4" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>T4</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="str">
+        <x:v>암호 4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="45" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>P4</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>T1</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D9" s="9" t="str">
+        <x:v>연결선 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="45" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>P4</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>T2</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="str">
+        <x:v>연결선 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="45" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>P4</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>T3</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D11" s="9" t="str">
+        <x:v>연결선 3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="45" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>P4</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>T4</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D12" s="9" t="str">
+        <x:v>연결선 4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="45" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>P7</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>T1</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="str">
+        <x:v>복원칸 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="45" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>P7</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>T2</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D14" s="9" t="str">
+        <x:v>복원칸 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="45" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>P7</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>T3</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D15" s="9" t="str">
+        <x:v>복원칸 3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="45" customHeight="1">
+      <x:c r="A16" s="4" t="str">
+        <x:v>P7</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>T4</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D16" s="9" t="str">
+        <x:v>복원칸 4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="45" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>P8</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>T1</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D17" s="9" t="str">
+        <x:v>열쇠홈 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="45" customHeight="1">
+      <x:c r="A18" s="4" t="str">
+        <x:v>P8</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>T2</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D18" s="9" t="str">
+        <x:v>열쇠홈 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="45" customHeight="1">
+      <x:c r="A19" s="4" t="str">
+        <x:v>P8</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>T3</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D19" s="9" t="str">
+        <x:v>열쇠홈 3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="45" customHeight="1">
+      <x:c r="A20" s="4" t="str">
+        <x:v>P8</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>T4</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>입력</x:v>
+      </x:c>
+      <x:c r="D20" s="9" t="str">
+        <x:v>열쇠홈 4</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1592,10 +2041,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>원본 기록</x:v>
+        <x:v>기록 1 · 윤재</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
-        <x:v>1번 다이얼: 둥근 테두리다. 안쪽이 비어 있고, 뾰족한 부분은 없다.</x:v>
+        <x:v>물의 분자식은 H₂O다. 원자 수가 두 개인 원소를 찾는다.</x:v>
       </x:c>
       <x:c r="E13" s="10"/>
     </x:row>
@@ -1607,10 +2056,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>설치 메모</x:v>
+        <x:v>기록 2 · 도하</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
-        <x:v>2번 다이얼: 세 변이 이어진 닫힌 도형이다.</x:v>
+        <x:v>이산화탄소의 분자식은 CO₂다. 원자 수가 한 개인 원소를 찾는다.</x:v>
       </x:c>
       <x:c r="E14" s="10"/>
     </x:row>
@@ -1622,10 +2071,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>현장 관찰</x:v>
+        <x:v>기록 3 · 시우</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>3번 다이얼: 밤하늘의 작은 별처럼 다섯 갈래로 뾰족하다.</x:v>
+        <x:v>분자식 O₂로 나타내는 기체를 이루는 원소를 찾는다.</x:v>
       </x:c>
       <x:c r="E15" s="10"/>
     </x:row>
@@ -1637,10 +2086,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>정리 전 사진</x:v>
+        <x:v>기록 4 · 민우</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
-        <x:v>4번 다이얼: 원의 한쪽이 크게 파인 밤하늘 모양이다.</x:v>
+        <x:v>분자식 N₂로 나타내는 기체를 이루는 원소를 찾는다.</x:v>
       </x:c>
       <x:c r="E16" s="10"/>
     </x:row>
@@ -1652,10 +2101,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>원본 기록</x:v>
+        <x:v>기록 1 · 윤재</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
-        <x:v>1번 선의 기록: 사람이 읽는 페이지 한 곳을 밝힌다.</x:v>
+        <x:v>입에서 침과 섞인 녹말이 분해되기 시작했다. 침 속에서 작용한 소화 효소는?</x:v>
       </x:c>
       <x:c r="E17" s="10"/>
     </x:row>
@@ -1667,10 +2116,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>설치 메모</x:v>
+        <x:v>기록 2 · 도하</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>2번 선의 기록: 실내 공기를 바깥으로 보낸다.</x:v>
+        <x:v>위에서 위액과 섞인 단백질이 분해되었다. 위액 속에서 작용한 소화 효소는?</x:v>
       </x:c>
       <x:c r="E18" s="10"/>
     </x:row>
@@ -1682,10 +2131,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>현장 관찰</x:v>
+        <x:v>기록 3 · 시우</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>3번 선의 기록: 목소리를 멀리 들려준다.</x:v>
+        <x:v>작은창자에서 이자액이 지방을 분해했다. 지방을 분해한 이자액 속 효소는?</x:v>
       </x:c>
       <x:c r="E19" s="10"/>
     </x:row>
@@ -1697,10 +2146,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>정리 전 사진</x:v>
+        <x:v>기록 4 · 민우</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>4번 선의 기록: 움직이는 빛이 아니라 글자로 소식을 전한다.</x:v>
+        <x:v>작은창자에서 이자액이 단백질을 분해했다. 단백질을 분해한 이자액 속 효소는?</x:v>
       </x:c>
       <x:c r="E20" s="10"/>
     </x:row>
@@ -1832,10 +2281,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>원본 기록</x:v>
+        <x:v>기록 1 · 윤재</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>1번 액자: 뿌리에서 막 올라온 작은 잎 두 장. 그림을 돌리지 않고 그대로 끼운다.</x:v>
+        <x:v>수소 원자 두 개가 결합한 분자 한 개의 모형.</x:v>
       </x:c>
       <x:c r="E29" s="10"/>
     </x:row>
@@ -1847,10 +2296,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>설치 메모</x:v>
+        <x:v>기록 2 · 도하</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
-        <x:v>2번 액자: 비를 막는 펼친 물건. 그림을 180° 돌려 거꾸로 끼운다.</x:v>
+        <x:v>수소 원자 두 개와 산소 원자 한 개가 결합한 분자 한 개의 모형.</x:v>
       </x:c>
       <x:c r="E30" s="10"/>
     </x:row>
@@ -1862,10 +2311,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C31" s="9" t="str">
-        <x:v>현장 관찰</x:v>
+        <x:v>기록 3 · 시우</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str">
-        <x:v>3번 액자: 눈을 뭉친 둥근 몸 두 개. 그림을 돌리지 않고 그대로 끼운다.</x:v>
+        <x:v>탄소 원자 한 개와 산소 원자 두 개가 결합한 분자 한 개의 모형.</x:v>
       </x:c>
       <x:c r="E31" s="10"/>
     </x:row>
@@ -1877,10 +2326,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>정리 전 사진</x:v>
+        <x:v>기록 4 · 민우</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>4번 액자: 나뭇가지에서 떨어진 잎 한 장. 그림을 180° 돌려 거꾸로 끼운다.</x:v>
+        <x:v>다른 원자와 결합하지 않은 헬륨 원자 한 개의 모형.</x:v>
       </x:c>
       <x:c r="E32" s="10"/>
     </x:row>
@@ -1892,10 +2341,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>원본 기록</x:v>
+        <x:v>기록 1 · 윤재</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
-        <x:v>1번 홈: 별 표식 조각. 화살표가 위로 향하는 앞면으로 끼운다.</x:v>
+        <x:v>위액이 나오는 기관. 단백질 소화가 시작되는 곳이다.</x:v>
       </x:c>
       <x:c r="E33" s="10"/>
     </x:row>
@@ -1907,10 +2356,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C34" s="9" t="str">
-        <x:v>설치 메모</x:v>
+        <x:v>기록 2 · 도하</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
-        <x:v>2번 홈: 원 표식 조각. 화살표가 아래로 향하도록 뒤집어 끼운다.</x:v>
+        <x:v>침과 음식물이 섞이는 기관. 씹어서 잘게 부수고 녹말 소화가 시작된다.</x:v>
       </x:c>
       <x:c r="E34" s="10"/>
     </x:row>
@@ -1922,10 +2371,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C35" s="9" t="str">
-        <x:v>현장 관찰</x:v>
+        <x:v>기록 3 · 시우</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
-        <x:v>3번 홈: 사각형 표식 조각. 화살표가 위로 향하는 앞면으로 끼운다.</x:v>
+        <x:v>안쪽 벽의 융털이 영양소를 흡수하는 기관.</x:v>
       </x:c>
       <x:c r="E35" s="10"/>
     </x:row>
@@ -1937,10 +2386,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C36" s="9" t="str">
-        <x:v>정리 전 사진</x:v>
+        <x:v>기록 4 · 민우</x:v>
       </x:c>
       <x:c r="D36" s="9" t="str">
-        <x:v>4번 홈: 삼각형 표식 조각. 화살표가 아래로 향하도록 뒤집어 끼운다.</x:v>
+        <x:v>대부분의 영양소가 흡수된 뒤 남은 내용물에서 수분을 더 흡수하고 대변을 만드는 기관.</x:v>
       </x:c>
       <x:c r="E36" s="10"/>
     </x:row>

</xml_diff>